<commit_message>
fix(marches): add bank support to marchés - update MarcheRequestDTO, MarcheResponseDTO, MarcheSearchDTO with banqueId and banqueNom - update MarcheInitializer to initialize banqueId when importing from XLSX
</commit_message>
<xml_diff>
--- a/gBanque/src/main/resources/marches_data.xlsx
+++ b/gBanque/src/main/resources/marches_data.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30794E52-D327-4696-A99C-D93D35FF8557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="783">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="792">
   <si>
     <t>numero</t>
   </si>
@@ -2363,13 +2369,40 @@
   </si>
   <si>
     <t>2023-12-12</t>
+  </si>
+  <si>
+    <t>Nom Banque</t>
+  </si>
+  <si>
+    <t>AWB</t>
+  </si>
+  <si>
+    <t>BMCE</t>
+  </si>
+  <si>
+    <t>BMCI</t>
+  </si>
+  <si>
+    <t>BP</t>
+  </si>
+  <si>
+    <t>CIH</t>
+  </si>
+  <si>
+    <t>CDM</t>
+  </si>
+  <si>
+    <t>SGMB</t>
+  </si>
+  <si>
+    <t>BPMG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2394,7 +2427,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2417,13 +2450,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -2432,13 +2479,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2476,7 +2531,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2510,6 +2565,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2544,9 +2600,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2719,11 +2776,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G201"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" customWidth="1"/>
+    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2742,8 +2808,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="2" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2751,7 +2820,7 @@
         <v>206</v>
       </c>
       <c r="C2">
-        <v>16472608.11</v>
+        <v>16472608.109999999</v>
       </c>
       <c r="D2" t="s">
         <v>406</v>
@@ -2762,8 +2831,11 @@
       <c r="F2" t="s">
         <v>599</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2771,7 +2843,7 @@
         <v>207</v>
       </c>
       <c r="C3">
-        <v>26598313.22</v>
+        <v>26598313.219999999</v>
       </c>
       <c r="D3" t="s">
         <v>407</v>
@@ -2782,8 +2854,11 @@
       <c r="F3" t="s">
         <v>600</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2791,7 +2866,7 @@
         <v>208</v>
       </c>
       <c r="C4">
-        <v>7239813.12</v>
+        <v>7239813.1200000001</v>
       </c>
       <c r="D4" t="s">
         <v>407</v>
@@ -2802,8 +2877,11 @@
       <c r="F4" t="s">
         <v>601</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2811,7 +2889,7 @@
         <v>209</v>
       </c>
       <c r="C5">
-        <v>7153556.95</v>
+        <v>7153556.9500000002</v>
       </c>
       <c r="D5" t="s">
         <v>406</v>
@@ -2822,8 +2900,11 @@
       <c r="F5" t="s">
         <v>602</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2831,7 +2912,7 @@
         <v>210</v>
       </c>
       <c r="C6">
-        <v>27182785.78</v>
+        <v>27182785.780000001</v>
       </c>
       <c r="D6" t="s">
         <v>408</v>
@@ -2842,8 +2923,11 @@
       <c r="F6" t="s">
         <v>603</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2851,7 +2935,7 @@
         <v>211</v>
       </c>
       <c r="C7">
-        <v>49652941.36</v>
+        <v>49652941.359999999</v>
       </c>
       <c r="D7" t="s">
         <v>409</v>
@@ -2862,8 +2946,11 @@
       <c r="F7" t="s">
         <v>604</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2871,7 +2958,7 @@
         <v>212</v>
       </c>
       <c r="C8">
-        <v>25915886.05</v>
+        <v>25915886.050000001</v>
       </c>
       <c r="D8" t="s">
         <v>408</v>
@@ -2882,8 +2969,11 @@
       <c r="F8" t="s">
         <v>605</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -2891,7 +2981,7 @@
         <v>213</v>
       </c>
       <c r="C9">
-        <v>24858330.81</v>
+        <v>24858330.809999999</v>
       </c>
       <c r="D9" t="s">
         <v>407</v>
@@ -2902,8 +2992,11 @@
       <c r="F9" t="s">
         <v>606</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -2922,8 +3015,11 @@
       <c r="F10" t="s">
         <v>607</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2931,7 +3027,7 @@
         <v>215</v>
       </c>
       <c r="C11">
-        <v>8735792.43</v>
+        <v>8735792.4299999997</v>
       </c>
       <c r="D11" t="s">
         <v>408</v>
@@ -2942,8 +3038,11 @@
       <c r="F11" t="s">
         <v>608</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2951,7 +3050,7 @@
         <v>216</v>
       </c>
       <c r="C12">
-        <v>27872091.72</v>
+        <v>27872091.719999999</v>
       </c>
       <c r="D12" t="s">
         <v>406</v>
@@ -2962,8 +3061,11 @@
       <c r="F12" t="s">
         <v>609</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -2971,7 +3073,7 @@
         <v>217</v>
       </c>
       <c r="C13">
-        <v>26197364.69</v>
+        <v>26197364.690000001</v>
       </c>
       <c r="D13" t="s">
         <v>406</v>
@@ -2982,8 +3084,11 @@
       <c r="F13" t="s">
         <v>610</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -2991,7 +3096,7 @@
         <v>218</v>
       </c>
       <c r="C14">
-        <v>34697307.71</v>
+        <v>34697307.710000001</v>
       </c>
       <c r="D14" t="s">
         <v>407</v>
@@ -3002,8 +3107,11 @@
       <c r="F14" t="s">
         <v>611</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -3022,8 +3130,11 @@
       <c r="F15" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -3031,7 +3142,7 @@
         <v>220</v>
       </c>
       <c r="C16">
-        <v>41451273.95</v>
+        <v>41451273.950000003</v>
       </c>
       <c r="D16" t="s">
         <v>408</v>
@@ -3042,8 +3153,11 @@
       <c r="F16" t="s">
         <v>613</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -3051,7 +3165,7 @@
         <v>221</v>
       </c>
       <c r="C17">
-        <v>26277141.67</v>
+        <v>26277141.670000002</v>
       </c>
       <c r="D17" t="s">
         <v>409</v>
@@ -3062,8 +3176,11 @@
       <c r="F17" t="s">
         <v>614</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -3071,7 +3188,7 @@
         <v>222</v>
       </c>
       <c r="C18">
-        <v>27434497.11</v>
+        <v>27434497.109999999</v>
       </c>
       <c r="D18" t="s">
         <v>410</v>
@@ -3082,8 +3199,11 @@
       <c r="F18" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -3091,7 +3211,7 @@
         <v>223</v>
       </c>
       <c r="C19">
-        <v>24403490.89</v>
+        <v>24403490.890000001</v>
       </c>
       <c r="D19" t="s">
         <v>407</v>
@@ -3102,8 +3222,11 @@
       <c r="F19" t="s">
         <v>616</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -3111,7 +3234,7 @@
         <v>224</v>
       </c>
       <c r="C20">
-        <v>43185977.67</v>
+        <v>43185977.670000002</v>
       </c>
       <c r="D20" t="s">
         <v>410</v>
@@ -3122,8 +3245,11 @@
       <c r="F20" t="s">
         <v>617</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -3131,7 +3257,7 @@
         <v>225</v>
       </c>
       <c r="C21">
-        <v>36123686.22</v>
+        <v>36123686.219999999</v>
       </c>
       <c r="D21" t="s">
         <v>407</v>
@@ -3142,8 +3268,11 @@
       <c r="F21" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -3151,7 +3280,7 @@
         <v>226</v>
       </c>
       <c r="C22">
-        <v>20959607.29</v>
+        <v>20959607.289999999</v>
       </c>
       <c r="D22" t="s">
         <v>407</v>
@@ -3162,8 +3291,11 @@
       <c r="F22" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -3171,7 +3303,7 @@
         <v>227</v>
       </c>
       <c r="C23">
-        <v>18928602.53</v>
+        <v>18928602.530000001</v>
       </c>
       <c r="D23" t="s">
         <v>408</v>
@@ -3182,8 +3314,11 @@
       <c r="F23" t="s">
         <v>620</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -3202,8 +3337,11 @@
       <c r="F24" t="s">
         <v>621</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -3211,7 +3349,7 @@
         <v>229</v>
       </c>
       <c r="C25">
-        <v>41371386.99</v>
+        <v>41371386.990000002</v>
       </c>
       <c r="D25" t="s">
         <v>409</v>
@@ -3222,8 +3360,11 @@
       <c r="F25" t="s">
         <v>622</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -3231,7 +3372,7 @@
         <v>230</v>
       </c>
       <c r="C26">
-        <v>38446255.85</v>
+        <v>38446255.850000001</v>
       </c>
       <c r="D26" t="s">
         <v>410</v>
@@ -3242,8 +3383,11 @@
       <c r="F26" t="s">
         <v>623</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -3251,7 +3395,7 @@
         <v>231</v>
       </c>
       <c r="C27">
-        <v>49722642.61</v>
+        <v>49722642.609999999</v>
       </c>
       <c r="D27" t="s">
         <v>409</v>
@@ -3262,8 +3406,11 @@
       <c r="F27" t="s">
         <v>624</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -3271,7 +3418,7 @@
         <v>232</v>
       </c>
       <c r="C28">
-        <v>32621367.29</v>
+        <v>32621367.289999999</v>
       </c>
       <c r="D28" t="s">
         <v>410</v>
@@ -3282,8 +3429,11 @@
       <c r="F28" t="s">
         <v>625</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -3302,8 +3452,11 @@
       <c r="F29" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -3311,7 +3464,7 @@
         <v>234</v>
       </c>
       <c r="C30">
-        <v>16927182.74</v>
+        <v>16927182.739999998</v>
       </c>
       <c r="D30" t="s">
         <v>407</v>
@@ -3322,8 +3475,11 @@
       <c r="F30" t="s">
         <v>627</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -3331,7 +3487,7 @@
         <v>235</v>
       </c>
       <c r="C31">
-        <v>40103659.13</v>
+        <v>40103659.130000003</v>
       </c>
       <c r="D31" t="s">
         <v>410</v>
@@ -3342,8 +3498,11 @@
       <c r="F31" t="s">
         <v>628</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="G31" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -3351,7 +3510,7 @@
         <v>236</v>
       </c>
       <c r="C32">
-        <v>21148489.22</v>
+        <v>21148489.219999999</v>
       </c>
       <c r="D32" t="s">
         <v>410</v>
@@ -3362,8 +3521,11 @@
       <c r="F32" t="s">
         <v>629</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -3371,7 +3533,7 @@
         <v>237</v>
       </c>
       <c r="C33">
-        <v>42816507.05</v>
+        <v>42816507.049999997</v>
       </c>
       <c r="D33" t="s">
         <v>410</v>
@@ -3382,8 +3544,11 @@
       <c r="F33" t="s">
         <v>630</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -3391,7 +3556,7 @@
         <v>238</v>
       </c>
       <c r="C34">
-        <v>11378389.11</v>
+        <v>11378389.109999999</v>
       </c>
       <c r="D34" t="s">
         <v>408</v>
@@ -3402,8 +3567,11 @@
       <c r="F34" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -3411,7 +3579,7 @@
         <v>239</v>
       </c>
       <c r="C35">
-        <v>44804120.94</v>
+        <v>44804120.939999998</v>
       </c>
       <c r="D35" t="s">
         <v>410</v>
@@ -3422,8 +3590,11 @@
       <c r="F35" t="s">
         <v>632</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -3442,8 +3613,11 @@
       <c r="F36" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -3451,7 +3625,7 @@
         <v>241</v>
       </c>
       <c r="C37">
-        <v>41604749.9</v>
+        <v>41604749.899999999</v>
       </c>
       <c r="D37" t="s">
         <v>409</v>
@@ -3462,8 +3636,11 @@
       <c r="F37" t="s">
         <v>634</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -3471,7 +3648,7 @@
         <v>242</v>
       </c>
       <c r="C38">
-        <v>32094134.62</v>
+        <v>32094134.620000001</v>
       </c>
       <c r="D38" t="s">
         <v>408</v>
@@ -3482,8 +3659,11 @@
       <c r="F38" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -3491,7 +3671,7 @@
         <v>243</v>
       </c>
       <c r="C39">
-        <v>30488749.51</v>
+        <v>30488749.510000002</v>
       </c>
       <c r="D39" t="s">
         <v>410</v>
@@ -3502,8 +3682,11 @@
       <c r="F39" t="s">
         <v>636</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -3522,8 +3705,11 @@
       <c r="F40" t="s">
         <v>637</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -3542,8 +3728,11 @@
       <c r="F41" t="s">
         <v>638</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -3562,8 +3751,11 @@
       <c r="F42" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -3582,8 +3774,11 @@
       <c r="F43" t="s">
         <v>640</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="G43" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -3591,7 +3786,7 @@
         <v>248</v>
       </c>
       <c r="C44">
-        <v>6893917.93</v>
+        <v>6893917.9299999997</v>
       </c>
       <c r="D44" t="s">
         <v>409</v>
@@ -3602,8 +3797,11 @@
       <c r="F44" t="s">
         <v>641</v>
       </c>
-    </row>
-    <row r="45" spans="1:6">
+      <c r="G44" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -3611,7 +3809,7 @@
         <v>249</v>
       </c>
       <c r="C45">
-        <v>16714423.8</v>
+        <v>16714423.800000001</v>
       </c>
       <c r="D45" t="s">
         <v>406</v>
@@ -3622,8 +3820,11 @@
       <c r="F45" t="s">
         <v>642</v>
       </c>
-    </row>
-    <row r="46" spans="1:6">
+      <c r="G45" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -3631,7 +3832,7 @@
         <v>250</v>
       </c>
       <c r="C46">
-        <v>11521198.62</v>
+        <v>11521198.619999999</v>
       </c>
       <c r="D46" t="s">
         <v>406</v>
@@ -3642,8 +3843,11 @@
       <c r="F46" t="s">
         <v>643</v>
       </c>
-    </row>
-    <row r="47" spans="1:6">
+      <c r="G46" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -3651,7 +3855,7 @@
         <v>251</v>
       </c>
       <c r="C47">
-        <v>29250674.78</v>
+        <v>29250674.780000001</v>
       </c>
       <c r="D47" t="s">
         <v>410</v>
@@ -3662,8 +3866,11 @@
       <c r="F47" t="s">
         <v>644</v>
       </c>
-    </row>
-    <row r="48" spans="1:6">
+      <c r="G47" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -3682,8 +3889,11 @@
       <c r="F48" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="49" spans="1:6">
+      <c r="G48" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -3702,8 +3912,11 @@
       <c r="F49" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="50" spans="1:6">
+      <c r="G49" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -3722,8 +3935,11 @@
       <c r="F50" t="s">
         <v>647</v>
       </c>
-    </row>
-    <row r="51" spans="1:6">
+      <c r="G50" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -3742,8 +3958,11 @@
       <c r="F51" t="s">
         <v>648</v>
       </c>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="G51" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -3751,7 +3970,7 @@
         <v>256</v>
       </c>
       <c r="C52">
-        <v>20160535.97</v>
+        <v>20160535.969999999</v>
       </c>
       <c r="D52" t="s">
         <v>410</v>
@@ -3762,8 +3981,11 @@
       <c r="F52" t="s">
         <v>649</v>
       </c>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="G52" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>57</v>
       </c>
@@ -3771,7 +3993,7 @@
         <v>257</v>
       </c>
       <c r="C53">
-        <v>31074373.9</v>
+        <v>31074373.899999999</v>
       </c>
       <c r="D53" t="s">
         <v>410</v>
@@ -3782,8 +4004,11 @@
       <c r="F53" t="s">
         <v>650</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="G53" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -3791,7 +4016,7 @@
         <v>258</v>
       </c>
       <c r="C54">
-        <v>45218016.58</v>
+        <v>45218016.579999998</v>
       </c>
       <c r="D54" t="s">
         <v>408</v>
@@ -3802,8 +4027,11 @@
       <c r="F54" t="s">
         <v>651</v>
       </c>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="G54" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -3811,7 +4039,7 @@
         <v>259</v>
       </c>
       <c r="C55">
-        <v>27999676.97</v>
+        <v>27999676.969999999</v>
       </c>
       <c r="D55" t="s">
         <v>409</v>
@@ -3822,8 +4050,11 @@
       <c r="F55" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="G55" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -3842,8 +4073,11 @@
       <c r="F56" t="s">
         <v>653</v>
       </c>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="G56" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>61</v>
       </c>
@@ -3851,7 +4085,7 @@
         <v>261</v>
       </c>
       <c r="C57">
-        <v>26861762.44</v>
+        <v>26861762.440000001</v>
       </c>
       <c r="D57" t="s">
         <v>408</v>
@@ -3862,8 +4096,11 @@
       <c r="F57" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="58" spans="1:6">
+      <c r="G57" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>62</v>
       </c>
@@ -3871,7 +4108,7 @@
         <v>262</v>
       </c>
       <c r="C58">
-        <v>46149528.47</v>
+        <v>46149528.469999999</v>
       </c>
       <c r="D58" t="s">
         <v>406</v>
@@ -3882,8 +4119,11 @@
       <c r="F58" t="s">
         <v>655</v>
       </c>
-    </row>
-    <row r="59" spans="1:6">
+      <c r="G58" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>63</v>
       </c>
@@ -3891,7 +4131,7 @@
         <v>263</v>
       </c>
       <c r="C59">
-        <v>32177746.26</v>
+        <v>32177746.260000002</v>
       </c>
       <c r="D59" t="s">
         <v>408</v>
@@ -3902,8 +4142,11 @@
       <c r="F59" t="s">
         <v>656</v>
       </c>
-    </row>
-    <row r="60" spans="1:6">
+      <c r="G59" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -3911,7 +4154,7 @@
         <v>264</v>
       </c>
       <c r="C60">
-        <v>8580853.07</v>
+        <v>8580853.0700000003</v>
       </c>
       <c r="D60" t="s">
         <v>409</v>
@@ -3922,8 +4165,11 @@
       <c r="F60" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="61" spans="1:6">
+      <c r="G60" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>65</v>
       </c>
@@ -3942,8 +4188,11 @@
       <c r="F61" t="s">
         <v>658</v>
       </c>
-    </row>
-    <row r="62" spans="1:6">
+      <c r="G61" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -3951,7 +4200,7 @@
         <v>266</v>
       </c>
       <c r="C62">
-        <v>28302607.12</v>
+        <v>28302607.120000001</v>
       </c>
       <c r="D62" t="s">
         <v>409</v>
@@ -3962,8 +4211,11 @@
       <c r="F62" t="s">
         <v>659</v>
       </c>
-    </row>
-    <row r="63" spans="1:6">
+      <c r="G62" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -3971,7 +4223,7 @@
         <v>267</v>
       </c>
       <c r="C63">
-        <v>4722408.15</v>
+        <v>4722408.1500000004</v>
       </c>
       <c r="D63" t="s">
         <v>408</v>
@@ -3982,8 +4234,11 @@
       <c r="F63" t="s">
         <v>660</v>
       </c>
-    </row>
-    <row r="64" spans="1:6">
+      <c r="G63" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -3991,7 +4246,7 @@
         <v>268</v>
       </c>
       <c r="C64">
-        <v>20302093.2</v>
+        <v>20302093.199999999</v>
       </c>
       <c r="D64" t="s">
         <v>407</v>
@@ -4002,8 +4257,11 @@
       <c r="F64" t="s">
         <v>661</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="G64" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -4011,7 +4269,7 @@
         <v>269</v>
       </c>
       <c r="C65">
-        <v>26007589.97</v>
+        <v>26007589.969999999</v>
       </c>
       <c r="D65" t="s">
         <v>406</v>
@@ -4022,8 +4280,11 @@
       <c r="F65" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="G65" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>70</v>
       </c>
@@ -4031,7 +4292,7 @@
         <v>270</v>
       </c>
       <c r="C66">
-        <v>38123361.59</v>
+        <v>38123361.590000004</v>
       </c>
       <c r="D66" t="s">
         <v>409</v>
@@ -4042,8 +4303,11 @@
       <c r="F66" t="s">
         <v>663</v>
       </c>
-    </row>
-    <row r="67" spans="1:6">
+      <c r="G66" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -4051,7 +4315,7 @@
         <v>271</v>
       </c>
       <c r="C67">
-        <v>7424396.38</v>
+        <v>7424396.3799999999</v>
       </c>
       <c r="D67" t="s">
         <v>406</v>
@@ -4062,8 +4326,11 @@
       <c r="F67" t="s">
         <v>664</v>
       </c>
-    </row>
-    <row r="68" spans="1:6">
+      <c r="G67" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>72</v>
       </c>
@@ -4071,7 +4338,7 @@
         <v>272</v>
       </c>
       <c r="C68">
-        <v>17338473.33</v>
+        <v>17338473.329999998</v>
       </c>
       <c r="D68" t="s">
         <v>406</v>
@@ -4082,8 +4349,11 @@
       <c r="F68" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="69" spans="1:6">
+      <c r="G68" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>73</v>
       </c>
@@ -4091,7 +4361,7 @@
         <v>273</v>
       </c>
       <c r="C69">
-        <v>44527209.7</v>
+        <v>44527209.700000003</v>
       </c>
       <c r="D69" t="s">
         <v>410</v>
@@ -4102,8 +4372,11 @@
       <c r="F69" t="s">
         <v>499</v>
       </c>
-    </row>
-    <row r="70" spans="1:6">
+      <c r="G69" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>74</v>
       </c>
@@ -4111,7 +4384,7 @@
         <v>274</v>
       </c>
       <c r="C70">
-        <v>46576943.49</v>
+        <v>46576943.490000002</v>
       </c>
       <c r="D70" t="s">
         <v>408</v>
@@ -4122,8 +4395,11 @@
       <c r="F70" t="s">
         <v>666</v>
       </c>
-    </row>
-    <row r="71" spans="1:6">
+      <c r="G70" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>75</v>
       </c>
@@ -4131,7 +4407,7 @@
         <v>275</v>
       </c>
       <c r="C71">
-        <v>26911659.69</v>
+        <v>26911659.690000001</v>
       </c>
       <c r="D71" t="s">
         <v>406</v>
@@ -4142,8 +4418,11 @@
       <c r="F71" t="s">
         <v>667</v>
       </c>
-    </row>
-    <row r="72" spans="1:6">
+      <c r="G71" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>76</v>
       </c>
@@ -4151,7 +4430,7 @@
         <v>276</v>
       </c>
       <c r="C72">
-        <v>21351171.56</v>
+        <v>21351171.559999999</v>
       </c>
       <c r="D72" t="s">
         <v>408</v>
@@ -4162,8 +4441,11 @@
       <c r="F72" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="73" spans="1:6">
+      <c r="G72" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>77</v>
       </c>
@@ -4182,8 +4464,11 @@
       <c r="F73" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="74" spans="1:6">
+      <c r="G73" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>78</v>
       </c>
@@ -4202,8 +4487,11 @@
       <c r="F74" t="s">
         <v>669</v>
       </c>
-    </row>
-    <row r="75" spans="1:6">
+      <c r="G74" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -4211,7 +4499,7 @@
         <v>279</v>
       </c>
       <c r="C75">
-        <v>34993900.4</v>
+        <v>34993900.399999999</v>
       </c>
       <c r="D75" t="s">
         <v>406</v>
@@ -4222,8 +4510,11 @@
       <c r="F75" t="s">
         <v>670</v>
       </c>
-    </row>
-    <row r="76" spans="1:6">
+      <c r="G75" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>80</v>
       </c>
@@ -4231,7 +4522,7 @@
         <v>280</v>
       </c>
       <c r="C76">
-        <v>30479274.99</v>
+        <v>30479274.989999998</v>
       </c>
       <c r="D76" t="s">
         <v>410</v>
@@ -4242,8 +4533,11 @@
       <c r="F76" t="s">
         <v>671</v>
       </c>
-    </row>
-    <row r="77" spans="1:6">
+      <c r="G76" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>81</v>
       </c>
@@ -4262,8 +4556,11 @@
       <c r="F77" t="s">
         <v>672</v>
       </c>
-    </row>
-    <row r="78" spans="1:6">
+      <c r="G77" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>82</v>
       </c>
@@ -4271,7 +4568,7 @@
         <v>282</v>
       </c>
       <c r="C78">
-        <v>37311718.23</v>
+        <v>37311718.229999997</v>
       </c>
       <c r="D78" t="s">
         <v>409</v>
@@ -4282,8 +4579,11 @@
       <c r="F78" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="79" spans="1:6">
+      <c r="G78" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -4291,7 +4591,7 @@
         <v>283</v>
       </c>
       <c r="C79">
-        <v>17038239.99</v>
+        <v>17038239.989999998</v>
       </c>
       <c r="D79" t="s">
         <v>406</v>
@@ -4302,8 +4602,11 @@
       <c r="F79" t="s">
         <v>495</v>
       </c>
-    </row>
-    <row r="80" spans="1:6">
+      <c r="G79" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>84</v>
       </c>
@@ -4311,7 +4614,7 @@
         <v>284</v>
       </c>
       <c r="C80">
-        <v>17695586.92</v>
+        <v>17695586.920000002</v>
       </c>
       <c r="D80" t="s">
         <v>409</v>
@@ -4322,8 +4625,11 @@
       <c r="F80" t="s">
         <v>674</v>
       </c>
-    </row>
-    <row r="81" spans="1:6">
+      <c r="G80" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>85</v>
       </c>
@@ -4342,8 +4648,11 @@
       <c r="F81" t="s">
         <v>675</v>
       </c>
-    </row>
-    <row r="82" spans="1:6">
+      <c r="G81" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>86</v>
       </c>
@@ -4351,7 +4660,7 @@
         <v>286</v>
       </c>
       <c r="C82">
-        <v>45550942.49</v>
+        <v>45550942.490000002</v>
       </c>
       <c r="D82" t="s">
         <v>406</v>
@@ -4362,8 +4671,11 @@
       <c r="F82" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="83" spans="1:6">
+      <c r="G82" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>87</v>
       </c>
@@ -4371,7 +4683,7 @@
         <v>287</v>
       </c>
       <c r="C83">
-        <v>26255248.69</v>
+        <v>26255248.690000001</v>
       </c>
       <c r="D83" t="s">
         <v>408</v>
@@ -4382,8 +4694,11 @@
       <c r="F83" t="s">
         <v>677</v>
       </c>
-    </row>
-    <row r="84" spans="1:6">
+      <c r="G83" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>88</v>
       </c>
@@ -4391,7 +4706,7 @@
         <v>288</v>
       </c>
       <c r="C84">
-        <v>4637681.65</v>
+        <v>4637681.6500000004</v>
       </c>
       <c r="D84" t="s">
         <v>408</v>
@@ -4402,8 +4717,11 @@
       <c r="F84" t="s">
         <v>678</v>
       </c>
-    </row>
-    <row r="85" spans="1:6">
+      <c r="G84" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>89</v>
       </c>
@@ -4411,7 +4729,7 @@
         <v>289</v>
       </c>
       <c r="C85">
-        <v>25091417.01</v>
+        <v>25091417.010000002</v>
       </c>
       <c r="D85" t="s">
         <v>410</v>
@@ -4422,8 +4740,11 @@
       <c r="F85" t="s">
         <v>679</v>
       </c>
-    </row>
-    <row r="86" spans="1:6">
+      <c r="G85" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>90</v>
       </c>
@@ -4442,8 +4763,11 @@
       <c r="F86" t="s">
         <v>596</v>
       </c>
-    </row>
-    <row r="87" spans="1:6">
+      <c r="G86" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>91</v>
       </c>
@@ -4462,8 +4786,11 @@
       <c r="F87" t="s">
         <v>680</v>
       </c>
-    </row>
-    <row r="88" spans="1:6">
+      <c r="G87" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>92</v>
       </c>
@@ -4471,7 +4798,7 @@
         <v>292</v>
       </c>
       <c r="C88">
-        <v>9297267.699999999</v>
+        <v>9297267.6999999993</v>
       </c>
       <c r="D88" t="s">
         <v>407</v>
@@ -4482,8 +4809,11 @@
       <c r="F88" t="s">
         <v>681</v>
       </c>
-    </row>
-    <row r="89" spans="1:6">
+      <c r="G88" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>93</v>
       </c>
@@ -4491,7 +4821,7 @@
         <v>293</v>
       </c>
       <c r="C89">
-        <v>18817784.1</v>
+        <v>18817784.100000001</v>
       </c>
       <c r="D89" t="s">
         <v>409</v>
@@ -4502,8 +4832,11 @@
       <c r="F89" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="90" spans="1:6">
+      <c r="G89" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>94</v>
       </c>
@@ -4511,7 +4844,7 @@
         <v>294</v>
       </c>
       <c r="C90">
-        <v>13734615.47</v>
+        <v>13734615.470000001</v>
       </c>
       <c r="D90" t="s">
         <v>409</v>
@@ -4522,8 +4855,11 @@
       <c r="F90" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="91" spans="1:6">
+      <c r="G90" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>95</v>
       </c>
@@ -4542,8 +4878,11 @@
       <c r="F91" t="s">
         <v>684</v>
       </c>
-    </row>
-    <row r="92" spans="1:6">
+      <c r="G91" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>96</v>
       </c>
@@ -4562,8 +4901,11 @@
       <c r="F92" t="s">
         <v>685</v>
       </c>
-    </row>
-    <row r="93" spans="1:6">
+      <c r="G92" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>97</v>
       </c>
@@ -4571,7 +4913,7 @@
         <v>297</v>
       </c>
       <c r="C93">
-        <v>22111172.19</v>
+        <v>22111172.190000001</v>
       </c>
       <c r="D93" t="s">
         <v>409</v>
@@ -4582,8 +4924,11 @@
       <c r="F93" t="s">
         <v>686</v>
       </c>
-    </row>
-    <row r="94" spans="1:6">
+      <c r="G93" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>98</v>
       </c>
@@ -4591,7 +4936,7 @@
         <v>298</v>
       </c>
       <c r="C94">
-        <v>47484748.04</v>
+        <v>47484748.039999999</v>
       </c>
       <c r="D94" t="s">
         <v>408</v>
@@ -4602,8 +4947,11 @@
       <c r="F94" t="s">
         <v>687</v>
       </c>
-    </row>
-    <row r="95" spans="1:6">
+      <c r="G94" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>99</v>
       </c>
@@ -4611,7 +4959,7 @@
         <v>299</v>
       </c>
       <c r="C95">
-        <v>13045779.06</v>
+        <v>13045779.060000001</v>
       </c>
       <c r="D95" t="s">
         <v>409</v>
@@ -4622,8 +4970,11 @@
       <c r="F95" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="96" spans="1:6">
+      <c r="G95" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>100</v>
       </c>
@@ -4631,7 +4982,7 @@
         <v>300</v>
       </c>
       <c r="C96">
-        <v>32146862.55</v>
+        <v>32146862.550000001</v>
       </c>
       <c r="D96" t="s">
         <v>407</v>
@@ -4642,8 +4993,11 @@
       <c r="F96" t="s">
         <v>689</v>
       </c>
-    </row>
-    <row r="97" spans="1:6">
+      <c r="G96" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>101</v>
       </c>
@@ -4651,7 +5005,7 @@
         <v>301</v>
       </c>
       <c r="C97">
-        <v>16614824.61</v>
+        <v>16614824.609999999</v>
       </c>
       <c r="D97" t="s">
         <v>406</v>
@@ -4662,8 +5016,11 @@
       <c r="F97" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="98" spans="1:6">
+      <c r="G97" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>102</v>
       </c>
@@ -4671,7 +5028,7 @@
         <v>302</v>
       </c>
       <c r="C98">
-        <v>49185867.1</v>
+        <v>49185867.100000001</v>
       </c>
       <c r="D98" t="s">
         <v>406</v>
@@ -4682,8 +5039,11 @@
       <c r="F98" t="s">
         <v>691</v>
       </c>
-    </row>
-    <row r="99" spans="1:6">
+      <c r="G98" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>103</v>
       </c>
@@ -4691,7 +5051,7 @@
         <v>303</v>
       </c>
       <c r="C99">
-        <v>15280075.78</v>
+        <v>15280075.779999999</v>
       </c>
       <c r="D99" t="s">
         <v>408</v>
@@ -4702,8 +5062,11 @@
       <c r="F99" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="100" spans="1:6">
+      <c r="G99" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>104</v>
       </c>
@@ -4711,7 +5074,7 @@
         <v>304</v>
       </c>
       <c r="C100">
-        <v>19751901.94</v>
+        <v>19751901.940000001</v>
       </c>
       <c r="D100" t="s">
         <v>408</v>
@@ -4722,8 +5085,11 @@
       <c r="F100" t="s">
         <v>693</v>
       </c>
-    </row>
-    <row r="101" spans="1:6">
+      <c r="G100" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>105</v>
       </c>
@@ -4731,7 +5097,7 @@
         <v>305</v>
       </c>
       <c r="C101">
-        <v>17034749.8</v>
+        <v>17034749.800000001</v>
       </c>
       <c r="D101" t="s">
         <v>408</v>
@@ -4742,8 +5108,11 @@
       <c r="F101" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="102" spans="1:6">
+      <c r="G101" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>106</v>
       </c>
@@ -4762,8 +5131,11 @@
       <c r="F102" t="s">
         <v>517</v>
       </c>
-    </row>
-    <row r="103" spans="1:6">
+      <c r="G102" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>107</v>
       </c>
@@ -4782,8 +5154,11 @@
       <c r="F103" t="s">
         <v>695</v>
       </c>
-    </row>
-    <row r="104" spans="1:6">
+      <c r="G103" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>108</v>
       </c>
@@ -4791,7 +5166,7 @@
         <v>308</v>
       </c>
       <c r="C104">
-        <v>9391678.970000001</v>
+        <v>9391678.9700000007</v>
       </c>
       <c r="D104" t="s">
         <v>406</v>
@@ -4802,8 +5177,11 @@
       <c r="F104" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="105" spans="1:6">
+      <c r="G104" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>109</v>
       </c>
@@ -4822,8 +5200,11 @@
       <c r="F105" t="s">
         <v>697</v>
       </c>
-    </row>
-    <row r="106" spans="1:6">
+      <c r="G105" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>110</v>
       </c>
@@ -4842,8 +5223,11 @@
       <c r="F106" t="s">
         <v>698</v>
       </c>
-    </row>
-    <row r="107" spans="1:6">
+      <c r="G106" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>111</v>
       </c>
@@ -4851,7 +5235,7 @@
         <v>311</v>
       </c>
       <c r="C107">
-        <v>13352376.14</v>
+        <v>13352376.140000001</v>
       </c>
       <c r="D107" t="s">
         <v>408</v>
@@ -4862,8 +5246,11 @@
       <c r="F107" t="s">
         <v>699</v>
       </c>
-    </row>
-    <row r="108" spans="1:6">
+      <c r="G107" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>112</v>
       </c>
@@ -4882,8 +5269,11 @@
       <c r="F108" t="s">
         <v>700</v>
       </c>
-    </row>
-    <row r="109" spans="1:6">
+      <c r="G108" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>113</v>
       </c>
@@ -4902,8 +5292,11 @@
       <c r="F109" t="s">
         <v>701</v>
       </c>
-    </row>
-    <row r="110" spans="1:6">
+      <c r="G109" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>114</v>
       </c>
@@ -4911,7 +5304,7 @@
         <v>314</v>
       </c>
       <c r="C110">
-        <v>31179924.65</v>
+        <v>31179924.649999999</v>
       </c>
       <c r="D110" t="s">
         <v>406</v>
@@ -4922,8 +5315,11 @@
       <c r="F110" t="s">
         <v>702</v>
       </c>
-    </row>
-    <row r="111" spans="1:6">
+      <c r="G110" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>115</v>
       </c>
@@ -4931,7 +5327,7 @@
         <v>315</v>
       </c>
       <c r="C111">
-        <v>41338396.31</v>
+        <v>41338396.310000002</v>
       </c>
       <c r="D111" t="s">
         <v>410</v>
@@ -4942,8 +5338,11 @@
       <c r="F111" t="s">
         <v>703</v>
       </c>
-    </row>
-    <row r="112" spans="1:6">
+      <c r="G111" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>116</v>
       </c>
@@ -4962,8 +5361,11 @@
       <c r="F112" t="s">
         <v>704</v>
       </c>
-    </row>
-    <row r="113" spans="1:6">
+      <c r="G112" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>117</v>
       </c>
@@ -4971,7 +5373,7 @@
         <v>317</v>
       </c>
       <c r="C113">
-        <v>7614447.82</v>
+        <v>7614447.8200000003</v>
       </c>
       <c r="D113" t="s">
         <v>406</v>
@@ -4982,8 +5384,11 @@
       <c r="F113" t="s">
         <v>705</v>
       </c>
-    </row>
-    <row r="114" spans="1:6">
+      <c r="G113" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>118</v>
       </c>
@@ -4991,7 +5396,7 @@
         <v>318</v>
       </c>
       <c r="C114">
-        <v>39754183.91</v>
+        <v>39754183.909999996</v>
       </c>
       <c r="D114" t="s">
         <v>407</v>
@@ -5002,8 +5407,11 @@
       <c r="F114" t="s">
         <v>706</v>
       </c>
-    </row>
-    <row r="115" spans="1:6">
+      <c r="G114" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>119</v>
       </c>
@@ -5011,7 +5419,7 @@
         <v>319</v>
       </c>
       <c r="C115">
-        <v>25020924.9</v>
+        <v>25020924.899999999</v>
       </c>
       <c r="D115" t="s">
         <v>407</v>
@@ -5022,8 +5430,11 @@
       <c r="F115" t="s">
         <v>707</v>
       </c>
-    </row>
-    <row r="116" spans="1:6">
+      <c r="G115" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>120</v>
       </c>
@@ -5031,7 +5442,7 @@
         <v>320</v>
       </c>
       <c r="C116">
-        <v>38215193.03</v>
+        <v>38215193.030000001</v>
       </c>
       <c r="D116" t="s">
         <v>408</v>
@@ -5042,8 +5453,11 @@
       <c r="F116" t="s">
         <v>708</v>
       </c>
-    </row>
-    <row r="117" spans="1:6">
+      <c r="G116" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>121</v>
       </c>
@@ -5062,8 +5476,11 @@
       <c r="F117" t="s">
         <v>709</v>
       </c>
-    </row>
-    <row r="118" spans="1:6">
+      <c r="G117" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>122</v>
       </c>
@@ -5071,7 +5488,7 @@
         <v>322</v>
       </c>
       <c r="C118">
-        <v>37783804.6</v>
+        <v>37783804.600000001</v>
       </c>
       <c r="D118" t="s">
         <v>410</v>
@@ -5082,8 +5499,11 @@
       <c r="F118" t="s">
         <v>710</v>
       </c>
-    </row>
-    <row r="119" spans="1:6">
+      <c r="G118" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>123</v>
       </c>
@@ -5091,7 +5511,7 @@
         <v>323</v>
       </c>
       <c r="C119">
-        <v>10421194.21</v>
+        <v>10421194.210000001</v>
       </c>
       <c r="D119" t="s">
         <v>408</v>
@@ -5102,8 +5522,11 @@
       <c r="F119" t="s">
         <v>711</v>
       </c>
-    </row>
-    <row r="120" spans="1:6">
+      <c r="G119" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>124</v>
       </c>
@@ -5111,7 +5534,7 @@
         <v>324</v>
       </c>
       <c r="C120">
-        <v>25772354.71</v>
+        <v>25772354.710000001</v>
       </c>
       <c r="D120" t="s">
         <v>406</v>
@@ -5122,8 +5545,11 @@
       <c r="F120" t="s">
         <v>667</v>
       </c>
-    </row>
-    <row r="121" spans="1:6">
+      <c r="G120" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>125</v>
       </c>
@@ -5131,7 +5557,7 @@
         <v>325</v>
       </c>
       <c r="C121">
-        <v>26106717.42</v>
+        <v>26106717.420000002</v>
       </c>
       <c r="D121" t="s">
         <v>409</v>
@@ -5142,8 +5568,11 @@
       <c r="F121" t="s">
         <v>712</v>
       </c>
-    </row>
-    <row r="122" spans="1:6">
+      <c r="G121" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>126</v>
       </c>
@@ -5151,7 +5580,7 @@
         <v>326</v>
       </c>
       <c r="C122">
-        <v>16925643.28</v>
+        <v>16925643.280000001</v>
       </c>
       <c r="D122" t="s">
         <v>406</v>
@@ -5162,8 +5591,11 @@
       <c r="F122" t="s">
         <v>713</v>
       </c>
-    </row>
-    <row r="123" spans="1:6">
+      <c r="G122" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>127</v>
       </c>
@@ -5171,7 +5603,7 @@
         <v>327</v>
       </c>
       <c r="C123">
-        <v>41279881.27</v>
+        <v>41279881.270000003</v>
       </c>
       <c r="D123" t="s">
         <v>408</v>
@@ -5182,8 +5614,11 @@
       <c r="F123" t="s">
         <v>714</v>
       </c>
-    </row>
-    <row r="124" spans="1:6">
+      <c r="G123" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>128</v>
       </c>
@@ -5202,8 +5637,11 @@
       <c r="F124" t="s">
         <v>715</v>
       </c>
-    </row>
-    <row r="125" spans="1:6">
+      <c r="G124" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>129</v>
       </c>
@@ -5211,7 +5649,7 @@
         <v>329</v>
       </c>
       <c r="C125">
-        <v>17511434.97</v>
+        <v>17511434.969999999</v>
       </c>
       <c r="D125" t="s">
         <v>407</v>
@@ -5222,8 +5660,11 @@
       <c r="F125" t="s">
         <v>716</v>
       </c>
-    </row>
-    <row r="126" spans="1:6">
+      <c r="G125" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>130</v>
       </c>
@@ -5242,8 +5683,11 @@
       <c r="F126" t="s">
         <v>717</v>
       </c>
-    </row>
-    <row r="127" spans="1:6">
+      <c r="G126" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>131</v>
       </c>
@@ -5251,7 +5695,7 @@
         <v>331</v>
       </c>
       <c r="C127">
-        <v>17051291.86</v>
+        <v>17051291.859999999</v>
       </c>
       <c r="D127" t="s">
         <v>407</v>
@@ -5262,8 +5706,11 @@
       <c r="F127" t="s">
         <v>718</v>
       </c>
-    </row>
-    <row r="128" spans="1:6">
+      <c r="G127" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>132</v>
       </c>
@@ -5271,7 +5718,7 @@
         <v>332</v>
       </c>
       <c r="C128">
-        <v>40474705.19</v>
+        <v>40474705.189999998</v>
       </c>
       <c r="D128" t="s">
         <v>408</v>
@@ -5282,8 +5729,11 @@
       <c r="F128" t="s">
         <v>719</v>
       </c>
-    </row>
-    <row r="129" spans="1:6">
+      <c r="G128" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>133</v>
       </c>
@@ -5302,8 +5752,11 @@
       <c r="F129" t="s">
         <v>720</v>
       </c>
-    </row>
-    <row r="130" spans="1:6">
+      <c r="G129" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>134</v>
       </c>
@@ -5311,7 +5764,7 @@
         <v>334</v>
       </c>
       <c r="C130">
-        <v>25154790.04</v>
+        <v>25154790.039999999</v>
       </c>
       <c r="D130" t="s">
         <v>406</v>
@@ -5322,8 +5775,11 @@
       <c r="F130" t="s">
         <v>721</v>
       </c>
-    </row>
-    <row r="131" spans="1:6">
+      <c r="G130" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>135</v>
       </c>
@@ -5331,7 +5787,7 @@
         <v>335</v>
       </c>
       <c r="C131">
-        <v>17343792.55</v>
+        <v>17343792.550000001</v>
       </c>
       <c r="D131" t="s">
         <v>409</v>
@@ -5342,8 +5798,11 @@
       <c r="F131" t="s">
         <v>722</v>
       </c>
-    </row>
-    <row r="132" spans="1:6">
+      <c r="G131" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>136</v>
       </c>
@@ -5351,7 +5810,7 @@
         <v>336</v>
       </c>
       <c r="C132">
-        <v>16478829.78</v>
+        <v>16478829.779999999</v>
       </c>
       <c r="D132" t="s">
         <v>408</v>
@@ -5362,8 +5821,11 @@
       <c r="F132" t="s">
         <v>723</v>
       </c>
-    </row>
-    <row r="133" spans="1:6">
+      <c r="G132" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>137</v>
       </c>
@@ -5371,7 +5833,7 @@
         <v>337</v>
       </c>
       <c r="C133">
-        <v>43442475.73</v>
+        <v>43442475.729999997</v>
       </c>
       <c r="D133" t="s">
         <v>407</v>
@@ -5382,8 +5844,11 @@
       <c r="F133" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="134" spans="1:6">
+      <c r="G133" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>138</v>
       </c>
@@ -5391,7 +5856,7 @@
         <v>338</v>
       </c>
       <c r="C134">
-        <v>7385895.2</v>
+        <v>7385895.2000000002</v>
       </c>
       <c r="D134" t="s">
         <v>409</v>
@@ -5402,8 +5867,11 @@
       <c r="F134" t="s">
         <v>724</v>
       </c>
-    </row>
-    <row r="135" spans="1:6">
+      <c r="G134" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>139</v>
       </c>
@@ -5411,7 +5879,7 @@
         <v>339</v>
       </c>
       <c r="C135">
-        <v>6302702.88</v>
+        <v>6302702.8799999999</v>
       </c>
       <c r="D135" t="s">
         <v>406</v>
@@ -5422,8 +5890,11 @@
       <c r="F135" t="s">
         <v>725</v>
       </c>
-    </row>
-    <row r="136" spans="1:6">
+      <c r="G135" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>140</v>
       </c>
@@ -5442,8 +5913,11 @@
       <c r="F136" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="137" spans="1:6">
+      <c r="G136" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>141</v>
       </c>
@@ -5451,7 +5925,7 @@
         <v>341</v>
       </c>
       <c r="C137">
-        <v>22205212.53</v>
+        <v>22205212.530000001</v>
       </c>
       <c r="D137" t="s">
         <v>410</v>
@@ -5462,8 +5936,11 @@
       <c r="F137" t="s">
         <v>727</v>
       </c>
-    </row>
-    <row r="138" spans="1:6">
+      <c r="G137" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>142</v>
       </c>
@@ -5482,8 +5959,11 @@
       <c r="F138" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="139" spans="1:6">
+      <c r="G138" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>143</v>
       </c>
@@ -5491,7 +5971,7 @@
         <v>343</v>
       </c>
       <c r="C139">
-        <v>11380611.03</v>
+        <v>11380611.029999999</v>
       </c>
       <c r="D139" t="s">
         <v>410</v>
@@ -5502,8 +5982,11 @@
       <c r="F139" t="s">
         <v>729</v>
       </c>
-    </row>
-    <row r="140" spans="1:6">
+      <c r="G139" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>144</v>
       </c>
@@ -5511,7 +5994,7 @@
         <v>344</v>
       </c>
       <c r="C140">
-        <v>13011706.71</v>
+        <v>13011706.710000001</v>
       </c>
       <c r="D140" t="s">
         <v>407</v>
@@ -5522,8 +6005,11 @@
       <c r="F140" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="141" spans="1:6">
+      <c r="G140" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>145</v>
       </c>
@@ -5531,7 +6017,7 @@
         <v>345</v>
       </c>
       <c r="C141">
-        <v>22147912.65</v>
+        <v>22147912.649999999</v>
       </c>
       <c r="D141" t="s">
         <v>406</v>
@@ -5542,8 +6028,11 @@
       <c r="F141" t="s">
         <v>731</v>
       </c>
-    </row>
-    <row r="142" spans="1:6">
+      <c r="G141" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>146</v>
       </c>
@@ -5551,7 +6040,7 @@
         <v>346</v>
       </c>
       <c r="C142">
-        <v>9060010.07</v>
+        <v>9060010.0700000003</v>
       </c>
       <c r="D142" t="s">
         <v>406</v>
@@ -5562,8 +6051,11 @@
       <c r="F142" t="s">
         <v>517</v>
       </c>
-    </row>
-    <row r="143" spans="1:6">
+      <c r="G142" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>147</v>
       </c>
@@ -5571,7 +6063,7 @@
         <v>347</v>
       </c>
       <c r="C143">
-        <v>21684542.96</v>
+        <v>21684542.960000001</v>
       </c>
       <c r="D143" t="s">
         <v>409</v>
@@ -5582,8 +6074,11 @@
       <c r="F143" t="s">
         <v>732</v>
       </c>
-    </row>
-    <row r="144" spans="1:6">
+      <c r="G143" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>148</v>
       </c>
@@ -5602,8 +6097,11 @@
       <c r="F144" t="s">
         <v>733</v>
       </c>
-    </row>
-    <row r="145" spans="1:6">
+      <c r="G144" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>149</v>
       </c>
@@ -5611,7 +6109,7 @@
         <v>349</v>
       </c>
       <c r="C145">
-        <v>43738133.48</v>
+        <v>43738133.479999997</v>
       </c>
       <c r="D145" t="s">
         <v>407</v>
@@ -5622,8 +6120,11 @@
       <c r="F145" t="s">
         <v>734</v>
       </c>
-    </row>
-    <row r="146" spans="1:6">
+      <c r="G145" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>150</v>
       </c>
@@ -5631,7 +6132,7 @@
         <v>350</v>
       </c>
       <c r="C146">
-        <v>4931182.94</v>
+        <v>4931182.9400000004</v>
       </c>
       <c r="D146" t="s">
         <v>406</v>
@@ -5642,8 +6143,11 @@
       <c r="F146" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="147" spans="1:6">
+      <c r="G146" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>151</v>
       </c>
@@ -5662,8 +6166,11 @@
       <c r="F147" t="s">
         <v>735</v>
       </c>
-    </row>
-    <row r="148" spans="1:6">
+      <c r="G147" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>152</v>
       </c>
@@ -5682,8 +6189,11 @@
       <c r="F148" t="s">
         <v>736</v>
       </c>
-    </row>
-    <row r="149" spans="1:6">
+      <c r="G148" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>153</v>
       </c>
@@ -5691,7 +6201,7 @@
         <v>353</v>
       </c>
       <c r="C149">
-        <v>35597778.31</v>
+        <v>35597778.310000002</v>
       </c>
       <c r="D149" t="s">
         <v>410</v>
@@ -5702,8 +6212,11 @@
       <c r="F149" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="150" spans="1:6">
+      <c r="G149" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>154</v>
       </c>
@@ -5711,7 +6224,7 @@
         <v>354</v>
       </c>
       <c r="C150">
-        <v>13225090.97</v>
+        <v>13225090.970000001</v>
       </c>
       <c r="D150" t="s">
         <v>408</v>
@@ -5722,8 +6235,11 @@
       <c r="F150" t="s">
         <v>738</v>
       </c>
-    </row>
-    <row r="151" spans="1:6">
+      <c r="G150" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>155</v>
       </c>
@@ -5742,8 +6258,11 @@
       <c r="F151" t="s">
         <v>739</v>
       </c>
-    </row>
-    <row r="152" spans="1:6">
+      <c r="G151" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>156</v>
       </c>
@@ -5751,7 +6270,7 @@
         <v>356</v>
       </c>
       <c r="C152">
-        <v>7209033.87</v>
+        <v>7209033.8700000001</v>
       </c>
       <c r="D152" t="s">
         <v>408</v>
@@ -5762,8 +6281,11 @@
       <c r="F152" t="s">
         <v>740</v>
       </c>
-    </row>
-    <row r="153" spans="1:6">
+      <c r="G152" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>157</v>
       </c>
@@ -5771,7 +6293,7 @@
         <v>357</v>
       </c>
       <c r="C153">
-        <v>27576225.19</v>
+        <v>27576225.190000001</v>
       </c>
       <c r="D153" t="s">
         <v>406</v>
@@ -5782,8 +6304,11 @@
       <c r="F153" t="s">
         <v>741</v>
       </c>
-    </row>
-    <row r="154" spans="1:6">
+      <c r="G153" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>158</v>
       </c>
@@ -5802,8 +6327,11 @@
       <c r="F154" t="s">
         <v>742</v>
       </c>
-    </row>
-    <row r="155" spans="1:6">
+      <c r="G154" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>159</v>
       </c>
@@ -5811,7 +6339,7 @@
         <v>359</v>
       </c>
       <c r="C155">
-        <v>19132504.26</v>
+        <v>19132504.260000002</v>
       </c>
       <c r="D155" t="s">
         <v>410</v>
@@ -5822,8 +6350,11 @@
       <c r="F155" t="s">
         <v>743</v>
       </c>
-    </row>
-    <row r="156" spans="1:6">
+      <c r="G155" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>160</v>
       </c>
@@ -5831,7 +6362,7 @@
         <v>360</v>
       </c>
       <c r="C156">
-        <v>49335203.19</v>
+        <v>49335203.189999998</v>
       </c>
       <c r="D156" t="s">
         <v>408</v>
@@ -5842,8 +6373,11 @@
       <c r="F156" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="157" spans="1:6">
+      <c r="G156" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>161</v>
       </c>
@@ -5851,7 +6385,7 @@
         <v>361</v>
       </c>
       <c r="C157">
-        <v>15864214.28</v>
+        <v>15864214.279999999</v>
       </c>
       <c r="D157" t="s">
         <v>409</v>
@@ -5862,8 +6396,11 @@
       <c r="F157" t="s">
         <v>745</v>
       </c>
-    </row>
-    <row r="158" spans="1:6">
+      <c r="G157" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>162</v>
       </c>
@@ -5871,7 +6408,7 @@
         <v>362</v>
       </c>
       <c r="C158">
-        <v>48699397.19</v>
+        <v>48699397.189999998</v>
       </c>
       <c r="D158" t="s">
         <v>409</v>
@@ -5882,8 +6419,11 @@
       <c r="F158" t="s">
         <v>746</v>
       </c>
-    </row>
-    <row r="159" spans="1:6">
+      <c r="G158" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>163</v>
       </c>
@@ -5891,7 +6431,7 @@
         <v>363</v>
       </c>
       <c r="C159">
-        <v>15186236.11</v>
+        <v>15186236.109999999</v>
       </c>
       <c r="D159" t="s">
         <v>407</v>
@@ -5902,8 +6442,11 @@
       <c r="F159" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="160" spans="1:6">
+      <c r="G159" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>164</v>
       </c>
@@ -5911,7 +6454,7 @@
         <v>364</v>
       </c>
       <c r="C160">
-        <v>1241339.85</v>
+        <v>1241339.8500000001</v>
       </c>
       <c r="D160" t="s">
         <v>407</v>
@@ -5922,8 +6465,11 @@
       <c r="F160" t="s">
         <v>747</v>
       </c>
-    </row>
-    <row r="161" spans="1:6">
+      <c r="G160" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>165</v>
       </c>
@@ -5931,7 +6477,7 @@
         <v>365</v>
       </c>
       <c r="C161">
-        <v>47286397.7</v>
+        <v>47286397.700000003</v>
       </c>
       <c r="D161" t="s">
         <v>409</v>
@@ -5942,8 +6488,11 @@
       <c r="F161" t="s">
         <v>748</v>
       </c>
-    </row>
-    <row r="162" spans="1:6">
+      <c r="G161" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>166</v>
       </c>
@@ -5951,7 +6500,7 @@
         <v>366</v>
       </c>
       <c r="C162">
-        <v>12371896.8</v>
+        <v>12371896.800000001</v>
       </c>
       <c r="D162" t="s">
         <v>407</v>
@@ -5962,8 +6511,11 @@
       <c r="F162" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="163" spans="1:6">
+      <c r="G162" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>167</v>
       </c>
@@ -5971,7 +6523,7 @@
         <v>367</v>
       </c>
       <c r="C163">
-        <v>47694112.1</v>
+        <v>47694112.100000001</v>
       </c>
       <c r="D163" t="s">
         <v>409</v>
@@ -5982,8 +6534,11 @@
       <c r="F163" t="s">
         <v>750</v>
       </c>
-    </row>
-    <row r="164" spans="1:6">
+      <c r="G163" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>168</v>
       </c>
@@ -5991,7 +6546,7 @@
         <v>368</v>
       </c>
       <c r="C164">
-        <v>42628378.05</v>
+        <v>42628378.049999997</v>
       </c>
       <c r="D164" t="s">
         <v>408</v>
@@ -6002,8 +6557,11 @@
       <c r="F164" t="s">
         <v>751</v>
       </c>
-    </row>
-    <row r="165" spans="1:6">
+      <c r="G164" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>169</v>
       </c>
@@ -6011,7 +6569,7 @@
         <v>369</v>
       </c>
       <c r="C165">
-        <v>24404395.6</v>
+        <v>24404395.600000001</v>
       </c>
       <c r="D165" t="s">
         <v>409</v>
@@ -6022,8 +6580,11 @@
       <c r="F165" t="s">
         <v>752</v>
       </c>
-    </row>
-    <row r="166" spans="1:6">
+      <c r="G165" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>170</v>
       </c>
@@ -6031,7 +6592,7 @@
         <v>370</v>
       </c>
       <c r="C166">
-        <v>37144734.1</v>
+        <v>37144734.100000001</v>
       </c>
       <c r="D166" t="s">
         <v>406</v>
@@ -6042,8 +6603,11 @@
       <c r="F166" t="s">
         <v>753</v>
       </c>
-    </row>
-    <row r="167" spans="1:6">
+      <c r="G166" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>171</v>
       </c>
@@ -6051,7 +6615,7 @@
         <v>371</v>
       </c>
       <c r="C167">
-        <v>11087472.61</v>
+        <v>11087472.609999999</v>
       </c>
       <c r="D167" t="s">
         <v>407</v>
@@ -6062,8 +6626,11 @@
       <c r="F167" t="s">
         <v>754</v>
       </c>
-    </row>
-    <row r="168" spans="1:6">
+      <c r="G167" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>172</v>
       </c>
@@ -6071,7 +6638,7 @@
         <v>372</v>
       </c>
       <c r="C168">
-        <v>15318035.88</v>
+        <v>15318035.880000001</v>
       </c>
       <c r="D168" t="s">
         <v>406</v>
@@ -6082,8 +6649,11 @@
       <c r="F168" t="s">
         <v>755</v>
       </c>
-    </row>
-    <row r="169" spans="1:6">
+      <c r="G168" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>173</v>
       </c>
@@ -6091,7 +6661,7 @@
         <v>373</v>
       </c>
       <c r="C169">
-        <v>26479677.47</v>
+        <v>26479677.469999999</v>
       </c>
       <c r="D169" t="s">
         <v>409</v>
@@ -6102,8 +6672,11 @@
       <c r="F169" t="s">
         <v>756</v>
       </c>
-    </row>
-    <row r="170" spans="1:6">
+      <c r="G169" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>174</v>
       </c>
@@ -6111,7 +6684,7 @@
         <v>374</v>
       </c>
       <c r="C170">
-        <v>42750221.84</v>
+        <v>42750221.840000004</v>
       </c>
       <c r="D170" t="s">
         <v>407</v>
@@ -6122,8 +6695,11 @@
       <c r="F170" t="s">
         <v>757</v>
       </c>
-    </row>
-    <row r="171" spans="1:6">
+      <c r="G170" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>175</v>
       </c>
@@ -6131,7 +6707,7 @@
         <v>375</v>
       </c>
       <c r="C171">
-        <v>16557959.39</v>
+        <v>16557959.390000001</v>
       </c>
       <c r="D171" t="s">
         <v>406</v>
@@ -6142,8 +6718,11 @@
       <c r="F171" t="s">
         <v>758</v>
       </c>
-    </row>
-    <row r="172" spans="1:6">
+      <c r="G171" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>176</v>
       </c>
@@ -6151,7 +6730,7 @@
         <v>376</v>
       </c>
       <c r="C172">
-        <v>48093900.86</v>
+        <v>48093900.859999999</v>
       </c>
       <c r="D172" t="s">
         <v>409</v>
@@ -6162,8 +6741,11 @@
       <c r="F172" t="s">
         <v>759</v>
       </c>
-    </row>
-    <row r="173" spans="1:6">
+      <c r="G172" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>177</v>
       </c>
@@ -6182,8 +6764,11 @@
       <c r="F173" t="s">
         <v>469</v>
       </c>
-    </row>
-    <row r="174" spans="1:6">
+      <c r="G173" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>178</v>
       </c>
@@ -6202,8 +6787,11 @@
       <c r="F174" t="s">
         <v>760</v>
       </c>
-    </row>
-    <row r="175" spans="1:6">
+      <c r="G174" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>179</v>
       </c>
@@ -6222,8 +6810,11 @@
       <c r="F175" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="176" spans="1:6">
+      <c r="G175" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>180</v>
       </c>
@@ -6231,7 +6822,7 @@
         <v>380</v>
       </c>
       <c r="C176">
-        <v>31886775.26</v>
+        <v>31886775.260000002</v>
       </c>
       <c r="D176" t="s">
         <v>408</v>
@@ -6242,8 +6833,11 @@
       <c r="F176" t="s">
         <v>761</v>
       </c>
-    </row>
-    <row r="177" spans="1:6">
+      <c r="G176" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>181</v>
       </c>
@@ -6251,7 +6845,7 @@
         <v>381</v>
       </c>
       <c r="C177">
-        <v>22834617.76</v>
+        <v>22834617.760000002</v>
       </c>
       <c r="D177" t="s">
         <v>407</v>
@@ -6262,8 +6856,11 @@
       <c r="F177" t="s">
         <v>762</v>
       </c>
-    </row>
-    <row r="178" spans="1:6">
+      <c r="G177" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>182</v>
       </c>
@@ -6271,7 +6868,7 @@
         <v>382</v>
       </c>
       <c r="C178">
-        <v>37770982.36</v>
+        <v>37770982.359999999</v>
       </c>
       <c r="D178" t="s">
         <v>407</v>
@@ -6282,8 +6879,11 @@
       <c r="F178" t="s">
         <v>763</v>
       </c>
-    </row>
-    <row r="179" spans="1:6">
+      <c r="G178" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>183</v>
       </c>
@@ -6291,7 +6891,7 @@
         <v>383</v>
       </c>
       <c r="C179">
-        <v>49813403.74</v>
+        <v>49813403.740000002</v>
       </c>
       <c r="D179" t="s">
         <v>409</v>
@@ -6302,8 +6902,11 @@
       <c r="F179" t="s">
         <v>764</v>
       </c>
-    </row>
-    <row r="180" spans="1:6">
+      <c r="G179" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>184</v>
       </c>
@@ -6311,7 +6914,7 @@
         <v>384</v>
       </c>
       <c r="C180">
-        <v>23930474.39</v>
+        <v>23930474.390000001</v>
       </c>
       <c r="D180" t="s">
         <v>406</v>
@@ -6322,8 +6925,11 @@
       <c r="F180" t="s">
         <v>765</v>
       </c>
-    </row>
-    <row r="181" spans="1:6">
+      <c r="G180" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>185</v>
       </c>
@@ -6342,8 +6948,11 @@
       <c r="F181" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="182" spans="1:6">
+      <c r="G181" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>186</v>
       </c>
@@ -6351,7 +6960,7 @@
         <v>386</v>
       </c>
       <c r="C182">
-        <v>35297208.04</v>
+        <v>35297208.039999999</v>
       </c>
       <c r="D182" t="s">
         <v>406</v>
@@ -6362,8 +6971,11 @@
       <c r="F182" t="s">
         <v>766</v>
       </c>
-    </row>
-    <row r="183" spans="1:6">
+      <c r="G182" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>187</v>
       </c>
@@ -6371,7 +6983,7 @@
         <v>387</v>
       </c>
       <c r="C183">
-        <v>37704833.06</v>
+        <v>37704833.060000002</v>
       </c>
       <c r="D183" t="s">
         <v>407</v>
@@ -6382,8 +6994,11 @@
       <c r="F183" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="184" spans="1:6">
+      <c r="G183" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>188</v>
       </c>
@@ -6391,7 +7006,7 @@
         <v>388</v>
       </c>
       <c r="C184">
-        <v>16744237.28</v>
+        <v>16744237.279999999</v>
       </c>
       <c r="D184" t="s">
         <v>406</v>
@@ -6402,8 +7017,11 @@
       <c r="F184" t="s">
         <v>767</v>
       </c>
-    </row>
-    <row r="185" spans="1:6">
+      <c r="G184" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>189</v>
       </c>
@@ -6411,7 +7029,7 @@
         <v>389</v>
       </c>
       <c r="C185">
-        <v>35881259.35</v>
+        <v>35881259.350000001</v>
       </c>
       <c r="D185" t="s">
         <v>407</v>
@@ -6422,8 +7040,11 @@
       <c r="F185" t="s">
         <v>768</v>
       </c>
-    </row>
-    <row r="186" spans="1:6">
+      <c r="G185" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>190</v>
       </c>
@@ -6431,7 +7052,7 @@
         <v>390</v>
       </c>
       <c r="C186">
-        <v>38181670.44</v>
+        <v>38181670.439999998</v>
       </c>
       <c r="D186" t="s">
         <v>408</v>
@@ -6442,8 +7063,11 @@
       <c r="F186" t="s">
         <v>769</v>
       </c>
-    </row>
-    <row r="187" spans="1:6">
+      <c r="G186" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>191</v>
       </c>
@@ -6451,7 +7075,7 @@
         <v>391</v>
       </c>
       <c r="C187">
-        <v>45879889.44</v>
+        <v>45879889.439999998</v>
       </c>
       <c r="D187" t="s">
         <v>410</v>
@@ -6462,8 +7086,11 @@
       <c r="F187" t="s">
         <v>605</v>
       </c>
-    </row>
-    <row r="188" spans="1:6">
+      <c r="G187" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>192</v>
       </c>
@@ -6482,8 +7109,11 @@
       <c r="F188" t="s">
         <v>701</v>
       </c>
-    </row>
-    <row r="189" spans="1:6">
+      <c r="G188" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>193</v>
       </c>
@@ -6502,8 +7132,11 @@
       <c r="F189" t="s">
         <v>770</v>
       </c>
-    </row>
-    <row r="190" spans="1:6">
+      <c r="G189" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>194</v>
       </c>
@@ -6511,7 +7144,7 @@
         <v>394</v>
       </c>
       <c r="C190">
-        <v>10680187.89</v>
+        <v>10680187.890000001</v>
       </c>
       <c r="D190" t="s">
         <v>410</v>
@@ -6522,8 +7155,11 @@
       <c r="F190" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="191" spans="1:6">
+      <c r="G190" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>195</v>
       </c>
@@ -6531,7 +7167,7 @@
         <v>395</v>
       </c>
       <c r="C191">
-        <v>29850171.35</v>
+        <v>29850171.350000001</v>
       </c>
       <c r="D191" t="s">
         <v>409</v>
@@ -6542,8 +7178,11 @@
       <c r="F191" t="s">
         <v>772</v>
       </c>
-    </row>
-    <row r="192" spans="1:6">
+      <c r="G191" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>196</v>
       </c>
@@ -6551,7 +7190,7 @@
         <v>396</v>
       </c>
       <c r="C192">
-        <v>22472284.79</v>
+        <v>22472284.789999999</v>
       </c>
       <c r="D192" t="s">
         <v>409</v>
@@ -6562,8 +7201,11 @@
       <c r="F192" t="s">
         <v>773</v>
       </c>
-    </row>
-    <row r="193" spans="1:6">
+      <c r="G192" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>197</v>
       </c>
@@ -6571,7 +7213,7 @@
         <v>397</v>
       </c>
       <c r="C193">
-        <v>29562073.86</v>
+        <v>29562073.859999999</v>
       </c>
       <c r="D193" t="s">
         <v>408</v>
@@ -6582,8 +7224,11 @@
       <c r="F193" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="194" spans="1:6">
+      <c r="G193" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>198</v>
       </c>
@@ -6591,7 +7236,7 @@
         <v>398</v>
       </c>
       <c r="C194">
-        <v>18516067.4</v>
+        <v>18516067.399999999</v>
       </c>
       <c r="D194" t="s">
         <v>410</v>
@@ -6602,8 +7247,11 @@
       <c r="F194" t="s">
         <v>775</v>
       </c>
-    </row>
-    <row r="195" spans="1:6">
+      <c r="G194" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>199</v>
       </c>
@@ -6611,7 +7259,7 @@
         <v>399</v>
       </c>
       <c r="C195">
-        <v>38761693.72</v>
+        <v>38761693.719999999</v>
       </c>
       <c r="D195" t="s">
         <v>409</v>
@@ -6622,8 +7270,11 @@
       <c r="F195" t="s">
         <v>776</v>
       </c>
-    </row>
-    <row r="196" spans="1:6">
+      <c r="G195" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>200</v>
       </c>
@@ -6642,8 +7293,11 @@
       <c r="F196" t="s">
         <v>777</v>
       </c>
-    </row>
-    <row r="197" spans="1:6">
+      <c r="G196" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>201</v>
       </c>
@@ -6651,7 +7305,7 @@
         <v>401</v>
       </c>
       <c r="C197">
-        <v>40034934.33</v>
+        <v>40034934.329999998</v>
       </c>
       <c r="D197" t="s">
         <v>410</v>
@@ -6662,8 +7316,11 @@
       <c r="F197" t="s">
         <v>778</v>
       </c>
-    </row>
-    <row r="198" spans="1:6">
+      <c r="G197" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>202</v>
       </c>
@@ -6671,7 +7328,7 @@
         <v>402</v>
       </c>
       <c r="C198">
-        <v>48588453.59</v>
+        <v>48588453.590000004</v>
       </c>
       <c r="D198" t="s">
         <v>407</v>
@@ -6682,8 +7339,11 @@
       <c r="F198" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="199" spans="1:6">
+      <c r="G198" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>203</v>
       </c>
@@ -6691,7 +7351,7 @@
         <v>403</v>
       </c>
       <c r="C199">
-        <v>13627732.04</v>
+        <v>13627732.039999999</v>
       </c>
       <c r="D199" t="s">
         <v>408</v>
@@ -6702,8 +7362,11 @@
       <c r="F199" t="s">
         <v>780</v>
       </c>
-    </row>
-    <row r="200" spans="1:6">
+      <c r="G199" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>204</v>
       </c>
@@ -6722,8 +7385,11 @@
       <c r="F200" t="s">
         <v>781</v>
       </c>
-    </row>
-    <row r="201" spans="1:6">
+      <c r="G200" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>205</v>
       </c>
@@ -6731,7 +7397,7 @@
         <v>405</v>
       </c>
       <c r="C201">
-        <v>45729569.52</v>
+        <v>45729569.520000003</v>
       </c>
       <c r="D201" t="s">
         <v>407</v>
@@ -6741,6 +7407,9 @@
       </c>
       <c r="F201" t="s">
         <v>782</v>
+      </c>
+      <c r="G201" t="s">
+        <v>786</v>
       </c>
     </row>
   </sheetData>

</xml_diff>